<commit_message>
docs: remove irrelavant sections and added requirement 3
</commit_message>
<xml_diff>
--- a/KCPM-HW01-Test Cases.xlsx
+++ b/KCPM-HW01-Test Cases.xlsx
@@ -113,9 +113,6 @@
   </si>
   <si>
     <t>Yes</t>
-  </si>
-  <si>
-    <t>Pending manual execution and video recording by student.</t>
   </si>
   <si>
     <t>Passed</t>
@@ -464,6 +461,9 @@
   </si>
   <si>
     <t>The grill prevents direct contact with rotating blades during normal use.</t>
+  </si>
+  <si>
+    <t>A finger-sized object can reach or make contact with the rotating blades through the grill opening.</t>
   </si>
   <si>
     <t>FAN-BUG-002</t>
@@ -1358,34 +1358,34 @@
         <v>30</v>
       </c>
       <c r="M3" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="N3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N3" s="13" t="s">
+      <c r="O3" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O3" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P3" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q3" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="R3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="R3" s="12" t="s">
+      <c r="S3" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T3" s="5"/>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="S3" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T3" s="5"/>
-    </row>
-    <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="9" t="s">
+      <c r="B4" s="10" t="s">
         <v>36</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>37</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>21</v>
@@ -1397,19 +1397,19 @@
         <v>23</v>
       </c>
       <c r="F4" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="G4" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="H4" s="11" t="s">
         <v>39</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>40</v>
       </c>
       <c r="I4" s="11" t="s">
         <v>27</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K4" s="11" t="s">
         <v>29</v>
@@ -1418,34 +1418,34 @@
         <v>30</v>
       </c>
       <c r="M4" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="N4" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N4" s="13" t="s">
+      <c r="O4" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O4" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P4" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q4" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R4" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="S4" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" s="5"/>
+    </row>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="S4" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T4" s="5"/>
-    </row>
-    <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="9" t="s">
+      <c r="B5" s="10" t="s">
         <v>43</v>
-      </c>
-      <c r="B5" s="10" t="s">
-        <v>44</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>21</v>
@@ -1457,19 +1457,19 @@
         <v>23</v>
       </c>
       <c r="F5" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="H5" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="11" t="s">
+      <c r="I5" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="11" t="s">
+      <c r="J5" s="11" t="s">
         <v>48</v>
-      </c>
-      <c r="J5" s="11" t="s">
-        <v>49</v>
       </c>
       <c r="K5" s="11" t="s">
         <v>29</v>
@@ -1478,34 +1478,34 @@
         <v>30</v>
       </c>
       <c r="M5" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="N5" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N5" s="13" t="s">
+      <c r="O5" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O5" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P5" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q5" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R5" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="S5" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T5" s="5"/>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="S5" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T5" s="5"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="9" t="s">
+      <c r="B6" s="10" t="s">
         <v>51</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>52</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>21</v>
@@ -1517,19 +1517,19 @@
         <v>23</v>
       </c>
       <c r="F6" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="H6" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="I6" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="J6" s="11" t="s">
         <v>56</v>
-      </c>
-      <c r="J6" s="11" t="s">
-        <v>57</v>
       </c>
       <c r="K6" s="11" t="s">
         <v>29</v>
@@ -1538,34 +1538,34 @@
         <v>30</v>
       </c>
       <c r="M6" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="N6" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N6" s="13" t="s">
+      <c r="O6" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O6" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P6" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q6" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R6" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="S6" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T6" s="5"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="S6" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T6" s="5"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="9" t="s">
+      <c r="B7" s="10" t="s">
         <v>59</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>60</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>21</v>
@@ -1577,19 +1577,19 @@
         <v>23</v>
       </c>
       <c r="F7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="G7" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="H7" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="I7" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="J7" s="11" t="s">
         <v>64</v>
-      </c>
-      <c r="J7" s="11" t="s">
-        <v>65</v>
       </c>
       <c r="K7" s="11" t="s">
         <v>29</v>
@@ -1598,34 +1598,34 @@
         <v>30</v>
       </c>
       <c r="M7" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="N7" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N7" s="13" t="s">
+      <c r="O7" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O7" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P7" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R7" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="S7" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T7" s="5"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="S7" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T7" s="5"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="9" t="s">
+      <c r="B8" s="10" t="s">
         <v>67</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>68</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>21</v>
@@ -1637,19 +1637,19 @@
         <v>23</v>
       </c>
       <c r="F8" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="G8" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="H8" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="H8" s="11" t="s">
-        <v>71</v>
-      </c>
       <c r="I8" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K8" s="11" t="s">
         <v>29</v>
@@ -1658,37 +1658,37 @@
         <v>30</v>
       </c>
       <c r="M8" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="N8" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N8" s="13" t="s">
+      <c r="O8" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O8" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P8" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q8" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R8" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="S8" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T8" s="5"/>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="S8" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T8" s="5"/>
-    </row>
-    <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="C9" s="10" t="s">
         <v>75</v>
-      </c>
-      <c r="C9" s="10" t="s">
-        <v>76</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>22</v>
@@ -1697,58 +1697,58 @@
         <v>23</v>
       </c>
       <c r="F9" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="J9" s="11" t="s">
         <v>80</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>81</v>
       </c>
       <c r="K9" s="11" t="s">
         <v>29</v>
       </c>
       <c r="L9" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="M9" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="M9" s="12" t="s">
+      <c r="N9" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="N9" s="12" t="s">
+      <c r="O9" s="12" t="s">
         <v>84</v>
-      </c>
-      <c r="O9" s="12" t="s">
-        <v>85</v>
       </c>
       <c r="P9" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q9" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R9" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="S9" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T9" s="5"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="S9" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T9" s="5"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C10" s="10" t="s">
         <v>88</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>89</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>22</v>
@@ -1757,19 +1757,19 @@
         <v>23</v>
       </c>
       <c r="F10" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="11" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="H10" s="11" t="s">
         <v>91</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="I10" s="11" t="s">
         <v>92</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="J10" s="11" t="s">
         <v>93</v>
-      </c>
-      <c r="J10" s="11" t="s">
-        <v>94</v>
       </c>
       <c r="K10" s="11" t="s">
         <v>29</v>
@@ -1778,37 +1778,37 @@
         <v>30</v>
       </c>
       <c r="M10" s="12" t="s">
+        <v>93</v>
+      </c>
+      <c r="N10" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N10" s="13" t="s">
+      <c r="O10" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O10" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P10" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q10" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R10" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="S10" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T10" s="5"/>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="S10" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T10" s="5"/>
-    </row>
-    <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="C11" s="10" t="s">
         <v>97</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>98</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>22</v>
@@ -1817,58 +1817,58 @@
         <v>23</v>
       </c>
       <c r="F11" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="G11" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="H11" s="11" t="s">
         <v>100</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="I11" s="11" t="s">
         <v>101</v>
       </c>
-      <c r="I11" s="11" t="s">
+      <c r="J11" s="11" t="s">
         <v>102</v>
-      </c>
-      <c r="J11" s="11" t="s">
-        <v>103</v>
       </c>
       <c r="K11" s="11" t="s">
         <v>29</v>
       </c>
       <c r="L11" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M11" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="N11" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N11" s="13" t="s">
+      <c r="O11" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O11" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P11" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q11" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R11" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="S11" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T11" s="5"/>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="S11" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T11" s="5"/>
-    </row>
-    <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>106</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>107</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>22</v>
@@ -1877,19 +1877,19 @@
         <v>23</v>
       </c>
       <c r="F12" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="G12" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="H12" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="I12" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="J12" s="11" t="s">
         <v>111</v>
-      </c>
-      <c r="J12" s="11" t="s">
-        <v>112</v>
       </c>
       <c r="K12" s="11" t="s">
         <v>29</v>
@@ -1898,37 +1898,37 @@
         <v>30</v>
       </c>
       <c r="M12" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="N12" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N12" s="13" t="s">
+      <c r="O12" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O12" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P12" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q12" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R12" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="S12" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T12" s="5"/>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="S12" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T12" s="5"/>
-    </row>
-    <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="C13" s="10" t="s">
         <v>115</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>116</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>22</v>
@@ -1937,19 +1937,19 @@
         <v>23</v>
       </c>
       <c r="F13" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="G13" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="H13" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="I13" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="J13" s="11" t="s">
         <v>120</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>121</v>
       </c>
       <c r="K13" s="11" t="s">
         <v>29</v>
@@ -1958,37 +1958,37 @@
         <v>30</v>
       </c>
       <c r="M13" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="N13" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N13" s="13" t="s">
+      <c r="O13" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O13" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P13" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q13" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R13" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="S13" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T13" s="5"/>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="S13" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T13" s="5"/>
-    </row>
-    <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="C14" s="10" t="s">
         <v>124</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="D14" s="10" t="s">
         <v>22</v>
@@ -1997,19 +1997,19 @@
         <v>23</v>
       </c>
       <c r="F14" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="G14" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="G14" s="11" t="s">
+      <c r="H14" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="I14" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="I14" s="11" t="s">
+      <c r="J14" s="11" t="s">
         <v>129</v>
-      </c>
-      <c r="J14" s="11" t="s">
-        <v>130</v>
       </c>
       <c r="K14" s="11" t="s">
         <v>29</v>
@@ -2018,37 +2018,37 @@
         <v>30</v>
       </c>
       <c r="M14" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="N14" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N14" s="13" t="s">
+      <c r="O14" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O14" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P14" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q14" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R14" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="S14" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="T14" s="5"/>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="S14" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="T14" s="5"/>
-    </row>
-    <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="C15" s="10" t="s">
         <v>133</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>134</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>22</v>
@@ -2057,19 +2057,19 @@
         <v>23</v>
       </c>
       <c r="F15" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="H15" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="G15" s="11" t="s">
-        <v>127</v>
-      </c>
-      <c r="H15" s="11" t="s">
+      <c r="I15" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="I15" s="11" t="s">
+      <c r="J15" s="11" t="s">
         <v>137</v>
-      </c>
-      <c r="J15" s="11" t="s">
-        <v>138</v>
       </c>
       <c r="K15" s="11" t="s">
         <v>29</v>
@@ -2077,11 +2077,11 @@
       <c r="L15" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="M15" s="12" t="s">
-        <v>31</v>
+      <c r="M15" s="13" t="s">
+        <v>138</v>
       </c>
       <c r="N15" s="13" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O15" s="13" t="s">
         <v>139</v>
@@ -2090,13 +2090,13 @@
         <v>29</v>
       </c>
       <c r="Q15" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R15" s="12" t="s">
         <v>140</v>
       </c>
       <c r="S15" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T15" s="5"/>
     </row>
@@ -2138,25 +2138,25 @@
         <v>30</v>
       </c>
       <c r="M16" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="N16" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N16" s="13" t="s">
+      <c r="O16" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O16" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P16" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q16" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R16" s="12" t="s">
         <v>149</v>
       </c>
       <c r="S16" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T16" s="5"/>
     </row>
@@ -2168,7 +2168,7 @@
         <v>151</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>22</v>
@@ -2180,7 +2180,7 @@
         <v>152</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>153</v>
@@ -2195,28 +2195,28 @@
         <v>29</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="M17" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="N17" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="N17" s="13" t="s">
+      <c r="O17" s="12" t="s">
         <v>32</v>
-      </c>
-      <c r="O17" s="12" t="s">
-        <v>33</v>
       </c>
       <c r="P17" s="12" t="s">
         <v>29</v>
       </c>
       <c r="Q17" s="14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="R17" s="12" t="s">
         <v>156</v>
       </c>
       <c r="S17" s="15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="T17" s="5"/>
     </row>
@@ -23994,7 +23994,7 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>167</v>
@@ -24006,10 +24006,10 @@
         <v>169</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G8" s="6" t="s">
         <v>170</v>
@@ -25165,7 +25165,7 @@
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B2" s="47" t="s">
         <v>178</v>
@@ -25237,7 +25237,7 @@
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="48" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" s="48" t="s">
         <v>183</v>
@@ -25273,7 +25273,7 @@
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="48" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B5" s="48" t="s">
         <v>185</v>
@@ -25309,7 +25309,7 @@
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="48" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B6" s="48" t="s">
         <v>187</v>
@@ -25345,7 +25345,7 @@
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="48" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B7" s="48" t="s">
         <v>189</v>
@@ -25381,7 +25381,7 @@
     </row>
     <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="48" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B8" s="48" t="s">
         <v>191</v>
@@ -25417,7 +25417,7 @@
     </row>
     <row r="9" ht="15.75" customHeight="1">
       <c r="A9" s="48" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B9" s="48" t="s">
         <v>193</v>
@@ -25453,7 +25453,7 @@
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="48" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B10" s="48" t="s">
         <v>195</v>
@@ -25489,7 +25489,7 @@
     </row>
     <row r="11" ht="15.75" customHeight="1">
       <c r="A11" s="48" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B11" s="48" t="s">
         <v>197</v>
@@ -25525,7 +25525,7 @@
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="48" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B12" s="48" t="s">
         <v>199</v>

</xml_diff>